<commit_message>
Cambios y más cambios
</commit_message>
<xml_diff>
--- a/Glosario.xlsx
+++ b/Glosario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8cd99136cfcc98d8/Documentos/FCFM/TesinaMCD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="8_{EC0D53CF-C172-4D0F-B149-549F69BA81B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAC3392C-AF20-4977-9736-533B17F2B94F}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{EC0D53CF-C172-4D0F-B149-549F69BA81B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62510E18-489B-4B21-81D1-58CB1FC99BF5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{D5830B11-BCB8-45B1-B10B-94BF0FDF060E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="105">
   <si>
     <t>Acrónimo</t>
   </si>
@@ -336,6 +336,21 @@
   </si>
   <si>
     <t>Punto de Rocío</t>
+  </si>
+  <si>
+    <t>CH</t>
+  </si>
+  <si>
+    <t>Calinski-Harabasz</t>
+  </si>
+  <si>
+    <t>BIC</t>
+  </si>
+  <si>
+    <t>criterio de información bayesiano</t>
+  </si>
+  <si>
+    <t>Bayesian Information Criterion</t>
   </si>
 </sst>
 </file>
@@ -581,10 +596,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA094194-6638-4829-AC95-20B12B18C431}" name="Table1" displayName="Table1" ref="A1:J39" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
-  <autoFilter ref="A1:J39" xr:uid="{CA094194-6638-4829-AC95-20B12B18C431}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J37">
-    <sortCondition ref="A1:A37"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CA094194-6638-4829-AC95-20B12B18C431}" name="Table1" displayName="Table1" ref="A1:J41" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+  <autoFilter ref="A1:J41" xr:uid="{CA094194-6638-4829-AC95-20B12B18C431}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:J39">
+    <sortCondition ref="A1:A39"/>
   </sortState>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{7F75F2B0-9B10-49A0-93D6-9E04264B5744}" name="Acrónimo" dataDxfId="9"/>
@@ -919,7 +934,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEA3C1E6-19F5-4F1D-A6FC-AD0154DC58E5}">
-  <dimension ref="A1:J39"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.6640625" style="1" customWidth="1"/>
@@ -1186,20 +1201,20 @@
     </row>
     <row r="12" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>45</v>
+        <v>98</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>46</v>
+        <v>99</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="str">
         <f>IF(A12="","",B12&amp;" ("&amp;IF(C12="","","\textit{"&amp;C12&amp;"}, ")&amp;A12&amp;")")</f>
-        <v>Gran Demanda en Baja Tensión (GDBT)</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>Punto de Rocío (DPT)</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -1207,15 +1222,15 @@
     </row>
     <row r="13" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>56</v>
+        <v>46</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="str">
         <f>IF(A13="","",B13&amp;" ("&amp;IF(C13="","","\textit{"&amp;C13&amp;"}, ")&amp;A13&amp;")")</f>
-        <v>gases de efecto invernadero (GEI)</v>
+        <v>Gran Demanda en Baja Tensión (GDBT)</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
@@ -1226,19 +1241,17 @@
       <c r="I13" s="2"/>
       <c r="J13" s="2"/>
     </row>
-    <row r="14" spans="1:10" ht="36" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>12</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="C14" s="2"/>
       <c r="D14" s="2" t="str">
         <f>IF(A14="","",B14&amp;" ("&amp;IF(C14="","","\textit{"&amp;C14&amp;"}, ")&amp;A14&amp;")")</f>
-        <v>Insituto de Redes de Energía Global (\textit{Global Energy Network Insitute}, GENI)</v>
+        <v>gases de efecto invernadero (GEI)</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
@@ -1249,19 +1262,19 @@
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
     </row>
-    <row r="15" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="36" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>72</v>
+        <v>11</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="D15" s="2" t="str">
         <f>IF(A15="","",B15&amp;" ("&amp;IF(C15="","","\textit{"&amp;C15&amp;"}, ")&amp;A15&amp;")")</f>
-        <v>modelo de mezcla gaussiana (\textit{Gaussian Mixture Model}, GMM)</v>
+        <v>Insituto de Redes de Energía Global (\textit{Global Energy Network Insitute}, GENI)</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2" t="s">
@@ -1274,19 +1287,21 @@
     </row>
     <row r="16" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D16" s="2" t="str">
         <f>IF(A16="","",B16&amp;" ("&amp;IF(C16="","","\textit{"&amp;C16&amp;"}, ")&amp;A16&amp;")")</f>
-        <v>regresión de procesos gaussianos (\textit{Gaussian Process Regression}, GPR)</v>
-      </c>
-      <c r="E16" s="2"/>
+        <v>modelo de mezcla gaussiana (\textit{Gaussian Mixture Model}, GMM)</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="F16" s="2" t="s">
         <v>24</v>
       </c>
@@ -1297,17 +1312,17 @@
     </row>
     <row r="17" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D17" s="2" t="str">
         <f>IF(A17="","",B17&amp;" ("&amp;IF(C17="","","\textit{"&amp;C17&amp;"}, ")&amp;A17&amp;")")</f>
-        <v>unidad recurrente con puertas (\textit{Gated Recurrent Unit}, GRU)</v>
+        <v>regresión de procesos gaussianos (\textit{Gaussian Process Regression}, GPR)</v>
       </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2" t="s">
@@ -1320,15 +1335,17 @@
     </row>
     <row r="18" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C18" s="2"/>
+        <v>82</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>83</v>
+      </c>
       <c r="D18" s="2" t="str">
         <f>IF(A18="","",B18&amp;" ("&amp;IF(C18="","","\textit{"&amp;C18&amp;"}, ")&amp;A18&amp;")")</f>
-        <v>Gigavatios-hora (GWh)</v>
+        <v>unidad recurrente con puertas (\textit{Gated Recurrent Unit}, GRU)</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2" t="s">
@@ -1341,15 +1358,15 @@
     </row>
     <row r="19" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2" t="str">
         <f>IF(A19="","",B19&amp;" ("&amp;IF(C19="","","\textit{"&amp;C19&amp;"}, ")&amp;A19&amp;")")</f>
-        <v>inteligencia artificial (IA)</v>
+        <v>Gigavatios-hora (GWh)</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2" t="s">
@@ -1360,63 +1377,63 @@
       <c r="I19" s="2"/>
       <c r="J19" s="2"/>
     </row>
-    <row r="20" spans="1:10" ht="36" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>3</v>
+        <v>59</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>5</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="C20" s="2"/>
       <c r="D20" s="2" t="str">
         <f>IF(A20="","",B20&amp;" ("&amp;IF(C20="","","\textit{"&amp;C20&amp;"}, ")&amp;A20&amp;")")</f>
-        <v>Grupo Intergubernamental de Expertos sobre el Cambio Climático (\textit{Intergovernmental Panel on Climate Change}, IPCC)</v>
+        <v>inteligencia artificial (IA)</v>
       </c>
       <c r="E20" s="2"/>
-      <c r="F20" s="2"/>
+      <c r="F20" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
-      <c r="J20" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="J20" s="2"/>
     </row>
     <row r="21" spans="1:10" ht="36" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D21" s="2" t="str">
         <f>IF(A21="","",B21&amp;" ("&amp;IF(C21="","","\textit{"&amp;C21&amp;"}, ")&amp;A21&amp;")")</f>
-        <v>Agencia Internacional de Energías Renovables (\textit{International Renewable Energy Agency}, IRENA)</v>
+        <v>Grupo Intergubernamental de Expertos sobre el Cambio Climático (\textit{Intergovernmental Panel on Climate Change}, IPCC)</v>
       </c>
       <c r="E21" s="2"/>
-      <c r="F21" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
-      <c r="J21" s="2"/>
-    </row>
-    <row r="22" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="J21" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="36" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C22" s="2"/>
+        <v>19</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>20</v>
+      </c>
       <c r="D22" s="2" t="str">
         <f>IF(A22="","",B22&amp;" ("&amp;IF(C22="","","\textit{"&amp;C22&amp;"}, ")&amp;A22&amp;")")</f>
-        <v>julios (J)</v>
+        <v>Agencia Internacional de Energías Renovables (\textit{International Renewable Energy Agency}, IRENA)</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2" t="s">
@@ -1429,20 +1446,20 @@
     </row>
     <row r="23" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>94</v>
+        <v>33</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>95</v>
+        <v>34</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2" t="str">
         <f>IF(A23="","",B23&amp;" ("&amp;IF(C23="","","\textit{"&amp;C23&amp;"}, ")&amp;A23&amp;")")</f>
-        <v>kilómetros por hora (km/h)</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F23" s="2"/>
+        <v>julios (J)</v>
+      </c>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
@@ -1450,20 +1467,20 @@
     </row>
     <row r="24" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>37</v>
+        <v>94</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>38</v>
+        <v>95</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2" t="str">
         <f>IF(A24="","",B24&amp;" ("&amp;IF(C24="","","\textit{"&amp;C24&amp;"}, ")&amp;A24&amp;")")</f>
-        <v>kilovatios (kW)</v>
-      </c>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>kilómetros por hora (km/h)</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
@@ -1471,19 +1488,17 @@
     </row>
     <row r="25" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2" t="str">
         <f>IF(A25="","",B25&amp;" ("&amp;IF(C25="","","\textit{"&amp;C25&amp;"}, ")&amp;A25&amp;")")</f>
-        <v>kilovatio-hora (kWh)</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>kilovatios (kW)</v>
+      </c>
+      <c r="E25" s="2"/>
       <c r="F25" s="2" t="s">
         <v>24</v>
       </c>
@@ -1494,19 +1509,19 @@
     </row>
     <row r="26" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>77</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="C26" s="2"/>
       <c r="D26" s="2" t="str">
         <f>IF(A26="","",B26&amp;" ("&amp;IF(C26="","","\textit{"&amp;C26&amp;"}, ")&amp;A26&amp;")")</f>
-        <v>memoria a largo  y corto plazo (\textit{Long Short-Term Network}, LSTM)</v>
-      </c>
-      <c r="E26" s="2"/>
+        <v>kilovatio-hora (kWh)</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="F26" s="2" t="s">
         <v>24</v>
       </c>
@@ -1517,22 +1532,22 @@
     </row>
     <row r="27" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
-        <v>88</v>
+        <v>63</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>89</v>
+        <v>64</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="D27" s="2" t="str">
         <f>IF(A27="","",B27&amp;" ("&amp;IF(C27="","","\textit{"&amp;C27&amp;"}, ")&amp;A27&amp;")")</f>
-        <v>error absoluto medio (\textit{Mean Absolute Error}, MAE)</v>
-      </c>
-      <c r="E27" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F27" s="2"/>
+        <v>memoria a largo  y corto plazo (\textit{Long Short-Term Network}, LSTM)</v>
+      </c>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="2"/>
@@ -1540,63 +1555,65 @@
     </row>
     <row r="28" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
-        <v>28</v>
+        <v>88</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C28" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="D28" s="2" t="str">
         <f>IF(A28="","",B28&amp;" ("&amp;IF(C28="","","\textit{"&amp;C28&amp;"}, ")&amp;A28&amp;")")</f>
-        <v>Mercado Eléctrico Mayorista (MEM)</v>
-      </c>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>error absoluto medio (\textit{Mean Absolute Error}, MAE)</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F28" s="2"/>
       <c r="G28" s="2"/>
-      <c r="H28" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
       <c r="J28" s="2"/>
     </row>
-    <row r="29" spans="1:10" ht="36" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>65</v>
+        <v>28</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>78</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="C29" s="2"/>
       <c r="D29" s="2" t="str">
         <f>IF(A29="","",B29&amp;" ("&amp;IF(C29="","","\textit{"&amp;C29&amp;"}, ")&amp;A29&amp;")")</f>
-        <v>optimizador de serpiente mejorado con estrategias múltiples (\textit{Multi-Strategy Improved Snake Optimizer}, MISO)</v>
+        <v>Mercado Eléctrico Mayorista (MEM)</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" s="2" t="s">
         <v>24</v>
       </c>
       <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
+      <c r="H29" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="J29" s="2"/>
     </row>
-    <row r="30" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="36" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>39</v>
+        <v>65</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C30" s="2"/>
+        <v>66</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="D30" s="2" t="str">
         <f>IF(A30="","",B30&amp;" ("&amp;IF(C30="","","\textit{"&amp;C30&amp;"}, ")&amp;A30&amp;")")</f>
-        <v>megavatios (MW)</v>
+        <v>optimizador de serpiente mejorado con estrategias múltiples (\textit{Multi-Strategy Improved Snake Optimizer}, MISO)</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" s="2" t="s">
@@ -1609,20 +1626,20 @@
     </row>
     <row r="31" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
-        <v>43</v>
+        <v>96</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>44</v>
+        <v>97</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2" t="str">
         <f>IF(A31="","",B31&amp;" ("&amp;IF(C31="","","\textit{"&amp;C31&amp;"}, ")&amp;A31&amp;")")</f>
-        <v>Pequeña Demanda en Baja Tensión (PDBT)</v>
-      </c>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>milímetros (mm)</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
@@ -1630,19 +1647,17 @@
     </row>
     <row r="32" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>68</v>
+        <v>40</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2" t="str">
         <f>IF(A32="","",B32&amp;" ("&amp;IF(C32="","","\textit{"&amp;C32&amp;"}, ")&amp;A32&amp;")")</f>
-        <v>coeficiente de determinación (R2)</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>megavatios (MW)</v>
+      </c>
+      <c r="E32" s="2"/>
       <c r="F32" s="2" t="s">
         <v>24</v>
       </c>
@@ -1653,21 +1668,17 @@
     </row>
     <row r="33" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
-        <v>69</v>
+        <v>43</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>79</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="C33" s="2"/>
       <c r="D33" s="2" t="str">
         <f>IF(A33="","",B33&amp;" ("&amp;IF(C33="","","\textit{"&amp;C33&amp;"}, ")&amp;A33&amp;")")</f>
-        <v>raíz del error cuadrático medio (\textit{Root Mean Square Error}, RMSE)</v>
-      </c>
-      <c r="E33" s="2" t="s">
-        <v>24</v>
-      </c>
+        <v>Pequeña Demanda en Baja Tensión (PDBT)</v>
+      </c>
+      <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
         <v>24</v>
       </c>
@@ -1678,19 +1689,19 @@
     </row>
     <row r="34" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>81</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="C34" s="2"/>
       <c r="D34" s="2" t="str">
         <f>IF(A34="","",B34&amp;" ("&amp;IF(C34="","","\textit{"&amp;C34&amp;"}, ")&amp;A34&amp;")")</f>
-        <v>redes neuronales recurrentes (\textit{Recurrent Neural Network}, RNN)</v>
-      </c>
-      <c r="E34" s="2"/>
+        <v>coeficiente de determinación (R2)</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="F34" s="2" t="s">
         <v>24</v>
       </c>
@@ -1701,40 +1712,42 @@
     </row>
     <row r="35" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
-        <v>7</v>
+        <v>69</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C35" s="2"/>
+        <v>70</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>79</v>
+      </c>
       <c r="D35" s="2" t="str">
         <f>IF(A35="","",B35&amp;" ("&amp;IF(C35="","","\textit{"&amp;C35&amp;"}, ")&amp;A35&amp;")")</f>
-        <v>Secretaría de Energía (SENER)</v>
-      </c>
-      <c r="E35" s="2"/>
+        <v>raíz del error cuadrático medio (\textit{Root Mean Square Error}, RMSE)</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="F35" s="2" t="s">
         <v>24</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
-      <c r="I35" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
     </row>
     <row r="36" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
-        <v>51</v>
+        <v>73</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C36" s="2"/>
+        <v>74</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="D36" s="2" t="str">
         <f>IF(A36="","",B36&amp;" ("&amp;IF(C36="","","\textit{"&amp;C36&amp;"}, ")&amp;A36&amp;")")</f>
-        <v>Suministrador de Servicios Básicos (SSB)</v>
+        <v>redes neuronales recurrentes (\textit{Recurrent Neural Network}, RNN)</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" s="2" t="s">
@@ -1745,17 +1758,17 @@
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
     </row>
-    <row r="37" spans="1:10" ht="36" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>54</v>
+        <v>8</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2" t="str">
         <f>IF(A37="","",B37&amp;" ("&amp;IF(C37="","","\textit{"&amp;C37&amp;"}, ")&amp;A37&amp;")")</f>
-        <v>Suministrador de Servicios Calificados (SSC)</v>
+        <v>Secretaría de Energía (SENER)</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="2" t="s">
@@ -1763,50 +1776,98 @@
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
-      <c r="I37" s="2"/>
-      <c r="J37" s="2"/>
+      <c r="I37" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="38" spans="1:10" ht="18" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>97</v>
+        <v>52</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2" t="str">
         <f>IF(A38="","",B38&amp;" ("&amp;IF(C38="","","\textit{"&amp;C38&amp;"}, ")&amp;A38&amp;")")</f>
-        <v>milímetros (mm)</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F38" s="2"/>
+        <v>Suministrador de Servicios Básicos (SSB)</v>
+      </c>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
     </row>
-    <row r="39" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" ht="36" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>99</v>
+        <v>54</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2" t="str">
         <f>IF(A39="","",B39&amp;" ("&amp;IF(C39="","","\textit{"&amp;C39&amp;"}, ")&amp;A39&amp;")")</f>
-        <v>Punto de Rocío (DPT)</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F39" s="2"/>
+        <v>Suministrador de Servicios Calificados (SSC)</v>
+      </c>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
+    </row>
+    <row r="40" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="A40" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2" t="str">
+        <f t="shared" ref="D40:D41" si="0">IF(A40="","",B40&amp;" ("&amp;IF(C40="","","\textit{"&amp;C40&amp;"}, ")&amp;A40&amp;")")</f>
+        <v>Calinski-Harabasz (CH)</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F40" s="2"/>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+    </row>
+    <row r="41" spans="1:10" ht="18" x14ac:dyDescent="0.35">
+      <c r="A41" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D41" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>criterio de información bayesiano (\textit{Bayesian Information Criterion}, BIC)</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>